<commit_message>
Refresh sample PDF/Excel from the final build
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SiP5Cz6QbE2dmCyYFoafBL
</commit_message>
<xml_diff>
--- a/docs/uat/samples/reports-all-sample-ar.xlsx
+++ b/docs/uat/samples/reports-all-sample-ar.xlsx
@@ -72,6 +72,9 @@
     <t>Nasir Hussain</t>
   </si>
   <si>
+    <t>Tariq Mahmood</t>
+  </si>
+  <si>
     <t>المهمة</t>
   </si>
   <si>
@@ -84,7 +87,7 @@
     <t>الاستحقاق التالي</t>
   </si>
   <si>
-    <t>Fertilizing</t>
+    <t>التسميد</t>
   </si>
   <si>
     <t>يحتاج متابعة</t>
@@ -120,10 +123,16 @@
     <t>مكتمل</t>
   </si>
   <si>
+    <t>#00002</t>
+  </si>
+  <si>
     <t>Sara</t>
   </si>
   <si>
     <t>قيد التنفيذ</t>
+  </si>
+  <si>
+    <t>#00001</t>
   </si>
 </sst>
 </file>
@@ -573,10 +582,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -587,7 +596,7 @@
         <v>46267</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -598,7 +607,7 @@
         <v>46267</v>
       </c>
       <c r="B10" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -609,7 +618,7 @@
         <v>46267</v>
       </c>
       <c r="B11" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -620,7 +629,7 @@
         <v>46267</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -631,7 +640,7 @@
         <v>46267</v>
       </c>
       <c r="B13" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -639,10 +648,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B14" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -650,10 +659,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="B15" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -664,7 +673,7 @@
         <v>46268</v>
       </c>
       <c r="B16" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -675,7 +684,7 @@
         <v>46268</v>
       </c>
       <c r="B17" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -686,7 +695,7 @@
         <v>46268</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -697,7 +706,7 @@
         <v>46268</v>
       </c>
       <c r="B19" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -705,10 +714,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2">
-        <v>46270</v>
+        <v>46268</v>
       </c>
       <c r="B20" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -716,10 +725,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2">
-        <v>46270</v>
+        <v>46268</v>
       </c>
       <c r="B21" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -727,10 +736,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2">
-        <v>46270</v>
+        <v>46268</v>
       </c>
       <c r="B22" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -741,7 +750,7 @@
         <v>46270</v>
       </c>
       <c r="B23" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -752,7 +761,7 @@
         <v>46270</v>
       </c>
       <c r="B24" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -763,7 +772,7 @@
         <v>46270</v>
       </c>
       <c r="B25" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -771,10 +780,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B26" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -782,10 +791,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B27" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -793,10 +802,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B28" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -804,10 +813,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B29" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -818,7 +827,7 @@
         <v>46271</v>
       </c>
       <c r="B30" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -829,7 +838,7 @@
         <v>46271</v>
       </c>
       <c r="B31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -837,10 +846,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B32" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -848,10 +857,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B33" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -859,10 +868,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -870,10 +879,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B35" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -881,10 +890,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B36" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -895,7 +904,7 @@
         <v>46272</v>
       </c>
       <c r="B37" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -903,10 +912,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B38" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -914,10 +923,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B39" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -925,10 +934,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C40">
         <v>1</v>
@@ -936,10 +945,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B41" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -947,10 +956,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B42" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C42">
         <v>1</v>
@@ -958,10 +967,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B43" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -969,7 +978,7 @@
     </row>
     <row r="44">
       <c r="A44" s="2">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B44" t="s">
         <v>7</v>
@@ -980,7 +989,7 @@
     </row>
     <row r="45">
       <c r="A45" s="2">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B45" t="s">
         <v>8</v>
@@ -991,7 +1000,7 @@
     </row>
     <row r="46">
       <c r="A46" s="2">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B46" t="s">
         <v>5</v>
@@ -1002,7 +1011,7 @@
     </row>
     <row r="47">
       <c r="A47" s="2">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B47" t="s">
         <v>3</v>
@@ -1013,7 +1022,7 @@
     </row>
     <row r="48">
       <c r="A48" s="2">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B48" t="s">
         <v>16</v>
@@ -1024,7 +1033,7 @@
     </row>
     <row r="49">
       <c r="A49" s="2">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>
@@ -1035,10 +1044,10 @@
     </row>
     <row r="50">
       <c r="A50" s="2">
-        <v>46275</v>
+        <v>46273</v>
       </c>
       <c r="B50" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -1046,10 +1055,10 @@
     </row>
     <row r="51">
       <c r="A51" s="2">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B51" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -1057,10 +1066,10 @@
     </row>
     <row r="52">
       <c r="A52" s="2">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B52" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -1068,10 +1077,10 @@
     </row>
     <row r="53">
       <c r="A53" s="2">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B53" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -1079,10 +1088,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B54" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -1090,10 +1099,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="B55" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C55">
         <v>1</v>
@@ -1101,10 +1110,10 @@
     </row>
     <row r="56">
       <c r="A56" s="2">
-        <v>46277</v>
+        <v>46274</v>
       </c>
       <c r="B56" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -1112,10 +1121,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2">
-        <v>46277</v>
+        <v>46274</v>
       </c>
       <c r="B57" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -1123,10 +1132,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="B58" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -1134,10 +1143,10 @@
     </row>
     <row r="59">
       <c r="A59" s="2">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="B59" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C59">
         <v>1</v>
@@ -1145,10 +1154,10 @@
     </row>
     <row r="60">
       <c r="A60" s="2">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="B60" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C60">
         <v>1</v>
@@ -1156,10 +1165,10 @@
     </row>
     <row r="61">
       <c r="A61" s="2">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="B61" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C61">
         <v>1</v>
@@ -1167,10 +1176,10 @@
     </row>
     <row r="62">
       <c r="A62" s="2">
-        <v>46278</v>
+        <v>46275</v>
       </c>
       <c r="B62" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C62">
         <v>1</v>
@@ -1178,10 +1187,10 @@
     </row>
     <row r="63">
       <c r="A63" s="2">
-        <v>46278</v>
+        <v>46275</v>
       </c>
       <c r="B63" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C63">
         <v>1</v>
@@ -1189,10 +1198,10 @@
     </row>
     <row r="64">
       <c r="A64" s="2">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B64" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C64">
         <v>1</v>
@@ -1200,10 +1209,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B65" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C65">
         <v>1</v>
@@ -1211,10 +1220,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B66" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C66">
         <v>1</v>
@@ -1222,10 +1231,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B67" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C67">
         <v>1</v>
@@ -1233,10 +1242,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="B68" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C68">
         <v>1</v>
@@ -1244,10 +1253,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="B69" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C69">
         <v>1</v>
@@ -1255,10 +1264,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B70" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -1266,10 +1275,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B71" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C71">
         <v>1</v>
@@ -1277,10 +1286,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B72" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C72">
         <v>1</v>
@@ -1288,10 +1297,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B73" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C73">
         <v>1</v>
@@ -1299,10 +1308,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2">
-        <v>46280</v>
+        <v>46278</v>
       </c>
       <c r="B74" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C74">
         <v>1</v>
@@ -1310,10 +1319,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2">
-        <v>46280</v>
+        <v>46278</v>
       </c>
       <c r="B75" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C75">
         <v>1</v>
@@ -1321,10 +1330,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B76" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C76">
         <v>1</v>
@@ -1332,10 +1341,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B77" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C77">
         <v>1</v>
@@ -1343,10 +1352,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B78" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C78">
         <v>1</v>
@@ -1354,10 +1363,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B79" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C79">
         <v>1</v>
@@ -1365,10 +1374,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="B80" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C80">
         <v>1</v>
@@ -1376,10 +1385,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="B81" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C81">
         <v>1</v>
@@ -1387,10 +1396,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B82" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C82">
         <v>1</v>
@@ -1398,10 +1407,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B83" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C83">
         <v>1</v>
@@ -1409,10 +1418,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B84" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C84">
         <v>1</v>
@@ -1420,10 +1429,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B85" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C85">
         <v>1</v>
@@ -1431,10 +1440,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2">
-        <v>46282</v>
+        <v>46280</v>
       </c>
       <c r="B86" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C86">
         <v>1</v>
@@ -1442,10 +1451,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2">
-        <v>46282</v>
+        <v>46280</v>
       </c>
       <c r="B87" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C87">
         <v>1</v>
@@ -1453,10 +1462,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B88" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C88">
         <v>1</v>
@@ -1464,10 +1473,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B89" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C89">
         <v>1</v>
@@ -1475,10 +1484,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B90" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C90">
         <v>1</v>
@@ -1486,10 +1495,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="B91" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C91">
         <v>1</v>
@@ -1497,10 +1506,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2">
-        <v>46284</v>
+        <v>46281</v>
       </c>
       <c r="B92" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C92">
         <v>1</v>
@@ -1508,10 +1517,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2">
-        <v>46284</v>
+        <v>46281</v>
       </c>
       <c r="B93" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C93">
         <v>1</v>
@@ -1519,10 +1528,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2">
-        <v>46284</v>
+        <v>46282</v>
       </c>
       <c r="B94" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C94">
         <v>1</v>
@@ -1530,10 +1539,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2">
-        <v>46284</v>
+        <v>46282</v>
       </c>
       <c r="B95" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C95">
         <v>1</v>
@@ -1541,10 +1550,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2">
-        <v>46284</v>
+        <v>46282</v>
       </c>
       <c r="B96" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C96">
         <v>1</v>
@@ -1552,10 +1561,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2">
-        <v>46284</v>
+        <v>46282</v>
       </c>
       <c r="B97" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C97">
         <v>1</v>
@@ -1563,10 +1572,10 @@
     </row>
     <row r="98">
       <c r="A98" s="2">
-        <v>46285</v>
+        <v>46282</v>
       </c>
       <c r="B98" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C98">
         <v>1</v>
@@ -1574,10 +1583,10 @@
     </row>
     <row r="99">
       <c r="A99" s="2">
-        <v>46285</v>
+        <v>46282</v>
       </c>
       <c r="B99" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C99">
         <v>1</v>
@@ -1585,10 +1594,10 @@
     </row>
     <row r="100">
       <c r="A100" s="2">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B100" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C100">
         <v>1</v>
@@ -1596,10 +1605,10 @@
     </row>
     <row r="101">
       <c r="A101" s="2">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B101" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C101">
         <v>1</v>
@@ -1607,10 +1616,10 @@
     </row>
     <row r="102">
       <c r="A102" s="2">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B102" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C102">
         <v>1</v>
@@ -1618,10 +1627,10 @@
     </row>
     <row r="103">
       <c r="A103" s="2">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B103" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C103">
         <v>1</v>
@@ -1629,10 +1638,10 @@
     </row>
     <row r="104">
       <c r="A104" s="2">
-        <v>46286</v>
+        <v>46284</v>
       </c>
       <c r="B104" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C104">
         <v>1</v>
@@ -1640,10 +1649,10 @@
     </row>
     <row r="105">
       <c r="A105" s="2">
-        <v>46286</v>
+        <v>46284</v>
       </c>
       <c r="B105" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C105">
         <v>1</v>
@@ -1651,10 +1660,10 @@
     </row>
     <row r="106">
       <c r="A106" s="2">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B106" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C106">
         <v>1</v>
@@ -1662,10 +1671,10 @@
     </row>
     <row r="107">
       <c r="A107" s="2">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B107" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C107">
         <v>1</v>
@@ -1673,10 +1682,10 @@
     </row>
     <row r="108">
       <c r="A108" s="2">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B108" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C108">
         <v>1</v>
@@ -1684,10 +1693,10 @@
     </row>
     <row r="109">
       <c r="A109" s="2">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B109" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C109">
         <v>1</v>
@@ -1695,10 +1704,10 @@
     </row>
     <row r="110">
       <c r="A110" s="2">
-        <v>46287</v>
+        <v>46285</v>
       </c>
       <c r="B110" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C110">
         <v>1</v>
@@ -1706,10 +1715,10 @@
     </row>
     <row r="111">
       <c r="A111" s="2">
-        <v>46287</v>
+        <v>46285</v>
       </c>
       <c r="B111" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C111">
         <v>1</v>
@@ -1717,10 +1726,10 @@
     </row>
     <row r="112">
       <c r="A112" s="2">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B112" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C112">
         <v>1</v>
@@ -1728,10 +1737,10 @@
     </row>
     <row r="113">
       <c r="A113" s="2">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B113" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C113">
         <v>1</v>
@@ -1739,10 +1748,10 @@
     </row>
     <row r="114">
       <c r="A114" s="2">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B114" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C114">
         <v>1</v>
@@ -1750,10 +1759,10 @@
     </row>
     <row r="115">
       <c r="A115" s="2">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="B115" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C115">
         <v>1</v>
@@ -1761,10 +1770,10 @@
     </row>
     <row r="116">
       <c r="A116" s="2">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="B116" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C116">
         <v>1</v>
@@ -1772,10 +1781,10 @@
     </row>
     <row r="117">
       <c r="A117" s="2">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="B117" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C117">
         <v>1</v>
@@ -1783,10 +1792,10 @@
     </row>
     <row r="118">
       <c r="A118" s="2">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B118" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C118">
         <v>1</v>
@@ -1794,10 +1803,10 @@
     </row>
     <row r="119">
       <c r="A119" s="2">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B119" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C119">
         <v>1</v>
@@ -1805,10 +1814,10 @@
     </row>
     <row r="120">
       <c r="A120" s="2">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B120" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C120">
         <v>1</v>
@@ -1816,10 +1825,10 @@
     </row>
     <row r="121">
       <c r="A121" s="2">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="B121" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C121">
         <v>1</v>
@@ -1827,10 +1836,10 @@
     </row>
     <row r="122">
       <c r="A122" s="2">
-        <v>46289</v>
+        <v>46287</v>
       </c>
       <c r="B122" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C122">
         <v>1</v>
@@ -1838,10 +1847,10 @@
     </row>
     <row r="123">
       <c r="A123" s="2">
-        <v>46289</v>
+        <v>46287</v>
       </c>
       <c r="B123" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C123">
         <v>1</v>
@@ -1849,10 +1858,10 @@
     </row>
     <row r="124">
       <c r="A124" s="2">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B124" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C124">
         <v>1</v>
@@ -1860,10 +1869,10 @@
     </row>
     <row r="125">
       <c r="A125" s="2">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B125" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C125">
         <v>1</v>
@@ -1871,10 +1880,10 @@
     </row>
     <row r="126">
       <c r="A126" s="2">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B126" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C126">
         <v>1</v>
@@ -1882,10 +1891,10 @@
     </row>
     <row r="127">
       <c r="A127" s="2">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="B127" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C127">
         <v>1</v>
@@ -1893,10 +1902,10 @@
     </row>
     <row r="128">
       <c r="A128" s="2">
-        <v>46291</v>
+        <v>46288</v>
       </c>
       <c r="B128" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C128">
         <v>1</v>
@@ -1904,10 +1913,10 @@
     </row>
     <row r="129">
       <c r="A129" s="2">
-        <v>46291</v>
+        <v>46288</v>
       </c>
       <c r="B129" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C129">
         <v>1</v>
@@ -1915,10 +1924,10 @@
     </row>
     <row r="130">
       <c r="A130" s="2">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="B130" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C130">
         <v>1</v>
@@ -1926,10 +1935,10 @@
     </row>
     <row r="131">
       <c r="A131" s="2">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="B131" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C131">
         <v>1</v>
@@ -1937,10 +1946,10 @@
     </row>
     <row r="132">
       <c r="A132" s="2">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="B132" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C132">
         <v>1</v>
@@ -1948,10 +1957,10 @@
     </row>
     <row r="133">
       <c r="A133" s="2">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="B133" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C133">
         <v>1</v>
@@ -1959,10 +1968,10 @@
     </row>
     <row r="134">
       <c r="A134" s="2">
-        <v>46292</v>
+        <v>46289</v>
       </c>
       <c r="B134" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C134">
         <v>1</v>
@@ -1970,10 +1979,10 @@
     </row>
     <row r="135">
       <c r="A135" s="2">
-        <v>46292</v>
+        <v>46289</v>
       </c>
       <c r="B135" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C135">
         <v>1</v>
@@ -1981,10 +1990,10 @@
     </row>
     <row r="136">
       <c r="A136" s="2">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B136" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C136">
         <v>1</v>
@@ -1992,10 +2001,10 @@
     </row>
     <row r="137">
       <c r="A137" s="2">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B137" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C137">
         <v>1</v>
@@ -2003,10 +2012,10 @@
     </row>
     <row r="138">
       <c r="A138" s="2">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B138" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C138">
         <v>1</v>
@@ -2014,10 +2023,10 @@
     </row>
     <row r="139">
       <c r="A139" s="2">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B139" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C139">
         <v>1</v>
@@ -2025,10 +2034,10 @@
     </row>
     <row r="140">
       <c r="A140" s="2">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="B140" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C140">
         <v>1</v>
@@ -2036,10 +2045,10 @@
     </row>
     <row r="141">
       <c r="A141" s="2">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="B141" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C141">
         <v>1</v>
@@ -2047,10 +2056,10 @@
     </row>
     <row r="142">
       <c r="A142" s="2">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B142" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C142">
         <v>1</v>
@@ -2058,10 +2067,10 @@
     </row>
     <row r="143">
       <c r="A143" s="2">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B143" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C143">
         <v>1</v>
@@ -2069,10 +2078,10 @@
     </row>
     <row r="144">
       <c r="A144" s="2">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B144" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C144">
         <v>1</v>
@@ -2080,10 +2089,10 @@
     </row>
     <row r="145">
       <c r="A145" s="2">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B145" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C145">
         <v>1</v>
@@ -2091,10 +2100,10 @@
     </row>
     <row r="146">
       <c r="A146" s="2">
-        <v>46294</v>
+        <v>46292</v>
       </c>
       <c r="B146" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C146">
         <v>1</v>
@@ -2102,21 +2111,21 @@
     </row>
     <row r="147">
       <c r="A147" s="2">
-        <v>46294</v>
+        <v>46292</v>
       </c>
       <c r="B147" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C147">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="B148" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C148">
         <v>1</v>
@@ -2124,10 +2133,10 @@
     </row>
     <row r="149">
       <c r="A149" s="2">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="B149" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C149">
         <v>1</v>
@@ -2135,10 +2144,10 @@
     </row>
     <row r="150">
       <c r="A150" s="2">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="B150" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C150">
         <v>1</v>
@@ -2146,18 +2155,18 @@
     </row>
     <row r="151">
       <c r="A151" s="2">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="B151" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C151">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="B152" t="s">
         <v>16</v>
@@ -2168,21 +2177,109 @@
     </row>
     <row r="153">
       <c r="A153" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B153" t="s">
+        <v>9</v>
+      </c>
+      <c r="C153">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B154" t="s">
+        <v>8</v>
+      </c>
+      <c r="C154">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B155" t="s">
+        <v>5</v>
+      </c>
+      <c r="C155">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B156" t="s">
+        <v>16</v>
+      </c>
+      <c r="C156">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2">
+        <v>46294</v>
+      </c>
+      <c r="B157" t="s">
+        <v>9</v>
+      </c>
+      <c r="C157">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2">
         <v>46295</v>
       </c>
-      <c r="B153" t="s">
-        <v>9</v>
-      </c>
-      <c r="C153">
+      <c r="B158" t="s">
+        <v>7</v>
+      </c>
+      <c r="C158">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B159" t="s">
+        <v>8</v>
+      </c>
+      <c r="C159">
         <v>0.5</v>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="1" t="s">
+    <row r="160">
+      <c r="A160" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B160" t="s">
+        <v>16</v>
+      </c>
+      <c r="C160">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2">
+        <v>46295</v>
+      </c>
+      <c r="B161" t="s">
+        <v>9</v>
+      </c>
+      <c r="C161">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C154" s="1">
-        <v>150.5</v>
+      <c r="C162" s="1">
+        <v>158.5</v>
       </c>
     </row>
   </sheetData>
@@ -2204,16 +2301,16 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2">
@@ -2221,13 +2318,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -2235,10 +2332,10 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -2246,10 +2343,10 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
         <v>26</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -2257,10 +2354,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -2280,7 +2377,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -2289,13 +2386,13 @@
         <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2">
@@ -2309,13 +2406,13 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
+        <v>33</v>
+      </c>
+      <c r="F2" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -2329,10 +2426,10 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
@@ -2346,13 +2443,13 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
+        <v>33</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix final regression findings and refresh evidence
- Nobody can change their own role (DB + UI); working-day changes audited
  (uuid-safe audit function)
- Same-named workers told apart in every filter and form
- Audit log: team/setup names, month formatted, empty changes hidden
- Correct Arabic and English plurals; day totals worded without plurals
- Visit checklist order stable across edits; small wording and layout fixes
- Evidence: 84 DB checks, 99 unit tests, regenerated samples

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SiP5Cz6QbE2dmCyYFoafBL
</commit_message>
<xml_diff>
--- a/docs/uat/samples/reports-all-sample-ar.xlsx
+++ b/docs/uat/samples/reports-all-sample-ar.xlsx
@@ -421,24 +421,24 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B2">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="D2">
-        <v>0.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4">

</xml_diff>